<commit_message>
added alot, pcb first prototype 4 layers
</commit_message>
<xml_diff>
--- a/parts.xlsx
+++ b/parts.xlsx
@@ -1,16 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reneb\Desktop\Bussysteme und Sensorik\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8556AE37-51B8-4D11-B5AF-CB63F9B06B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -20,108 +25,111 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
-  <si>
-    <t xml:space="preserve">Quant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PartName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MnfNo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DigikeyNo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP32-S3-WROOM-1-N8R2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5407-ESP32-S3-WROOM-1-N8R2-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.de/de/products/detail/espressif-systems/ESP32-S3-WROOM-1-N8R2/15200058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMS1117-3.3 SOT-223</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5399-AMS1117-3.3SOT-223CT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.de/de/products/detail/shenzhen-slkormicro-semicon-co-ltd/AMS1117-3-3-SOT-223/21853079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BMP390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">828-BMP390CT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.de/de/products/detail/bosch-sensortec/BMP390/16164577</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LM75BD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LM75BD,118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">568-4688-1-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.de/de/products/detail/nxp-usa-inc/LM75BD-118/1992993</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHTC3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHTC3-TR-2.5KS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1649-SHTC3-TR-2.5KSCT-ND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.digikey.de/de/products/detail/sensirion-ag/SHTC3-TR-2-5KS/8628148</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
+  <si>
+    <t>Quant</t>
+  </si>
+  <si>
+    <t>PartName</t>
+  </si>
+  <si>
+    <t>MnfNo.</t>
+  </si>
+  <si>
+    <t>DigikeyNo.</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>ESP32-S3-WROOM-1-N8R2</t>
+  </si>
+  <si>
+    <t>5407-ESP32-S3-WROOM-1-N8R2-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/espressif-systems/ESP32-S3-WROOM-1-N8R2/15200058</t>
+  </si>
+  <si>
+    <t>AMS1117-3.3 SOT-223</t>
+  </si>
+  <si>
+    <t>5399-AMS1117-3.3SOT-223CT-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/shenzhen-slkormicro-semicon-co-ltd/AMS1117-3-3-SOT-223/21853079</t>
+  </si>
+  <si>
+    <t>BMP390</t>
+  </si>
+  <si>
+    <t>828-BMP390CT-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/bosch-sensortec/BMP390/16164577</t>
+  </si>
+  <si>
+    <t>LM75BD</t>
+  </si>
+  <si>
+    <t>LM75BD,118</t>
+  </si>
+  <si>
+    <t>568-4688-1-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/nxp-usa-inc/LM75BD-118/1992993</t>
+  </si>
+  <si>
+    <t>SHTC3</t>
+  </si>
+  <si>
+    <t>SHTC3-TR-2.5KS</t>
+  </si>
+  <si>
+    <t>1649-SHTC3-TR-2.5KSCT-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/sensirion-ag/SHTC3-TR-2-5KS/8628148</t>
+  </si>
+  <si>
+    <t>296-26073-1-ND</t>
+  </si>
+  <si>
+    <t>INA219AIDCNT</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/texas-instruments/INA219AIDCNT/2047417</t>
+  </si>
+  <si>
+    <t>900-2171750001CT-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/molex/2171750001/13913745</t>
+  </si>
+  <si>
+    <t>https://www.digikey.de/de/products/detail/bosch-sensortec/BMP390/16164575</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00&quot; €&quot;;[RED]\-#,##0.00&quot; €&quot;"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00\ [$€-407];[RED]\-#,##0.00\ [$€-407]"/>
+    <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; €&quot;;[Red]\-#,##0.00&quot; €&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00\ [$€-407];[Red]\-#,##0.00\ [$€-407]"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -131,7 +139,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Bahnschrift Light"/>
@@ -139,7 +147,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
+      <u/>
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
@@ -168,7 +176,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -176,77 +184,34 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -305,60 +270,76 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -390,7 +371,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -414,7 +395,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -474,30 +455,29 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="110.6"/>
+    <col min="2" max="2" width="35.88671875" customWidth="1"/>
+    <col min="3" max="3" width="26.88671875" customWidth="1"/>
+    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="110.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,8 +497,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -530,15 +510,15 @@
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="4">
         <v>4.8</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -550,15 +530,15 @@
       <c r="D3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="4">
         <v>0.09</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -570,15 +550,15 @@
       <c r="D4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="E4" s="7">
         <v>2.68</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
@@ -590,15 +570,15 @@
       <c r="D5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="7">
         <v>0.5</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
         <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
@@ -610,46 +590,94 @@
       <c r="D6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="7">
         <v>1.76</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="8">
+        <v>2.27</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8" s="9">
+        <v>2171750001</v>
+      </c>
+      <c r="C8" s="10">
+        <v>2171750001</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="8">
+        <v>0.64</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="8">
+        <v>2.7</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="8">
+        <v>0.51</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="6"/>
       <c r="C11" s="1"/>
@@ -657,7 +685,7 @@
       <c r="E11" s="1"/>
       <c r="F11" s="6"/>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="6"/>
       <c r="C12" s="1"/>
@@ -665,7 +693,7 @@
       <c r="E12" s="1"/>
       <c r="F12" s="6"/>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="6"/>
       <c r="C13" s="1"/>
@@ -673,7 +701,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="6"/>
       <c r="C14" s="1"/>
@@ -681,7 +709,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
       <c r="C15" s="1"/>
@@ -689,7 +717,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="6"/>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
       <c r="C16" s="1"/>
@@ -697,7 +725,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="6"/>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
       <c r="C17" s="1"/>
@@ -705,7 +733,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="6"/>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
       <c r="C18" s="1"/>
@@ -713,7 +741,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="6"/>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
       <c r="C19" s="1"/>
@@ -721,7 +749,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="6"/>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
       <c r="C20" s="1"/>
@@ -729,7 +757,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="6"/>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="6"/>
       <c r="C21" s="1"/>
@@ -737,7 +765,7 @@
       <c r="E21" s="1"/>
       <c r="F21" s="6"/>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="6"/>
       <c r="C22" s="1"/>
@@ -745,7 +773,7 @@
       <c r="E22" s="1"/>
       <c r="F22" s="6"/>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="6"/>
       <c r="C23" s="1"/>
@@ -753,7 +781,7 @@
       <c r="E23" s="1"/>
       <c r="F23" s="6"/>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="6"/>
       <c r="C24" s="1"/>
@@ -761,7 +789,7 @@
       <c r="E24" s="1"/>
       <c r="F24" s="6"/>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="6"/>
       <c r="C25" s="1"/>
@@ -769,7 +797,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="6"/>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="6"/>
       <c r="C26" s="1"/>
@@ -777,7 +805,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="6"/>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="6"/>
       <c r="C27" s="1"/>
@@ -787,18 +815,15 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="https://www.digikey.de/de/products/detail/espressif-systems/ESP32-S3-WROOM-1-N8R2/15200058"/>
-    <hyperlink ref="F3" r:id="rId2" display="https://www.digikey.de/de/products/detail/shenzhen-slkormicro-semicon-co-ltd/AMS1117-3-3-SOT-223/21853079"/>
-    <hyperlink ref="F4" r:id="rId3" display="https://www.digikey.de/de/products/detail/bosch-sensortec/BMP390/16164577"/>
-    <hyperlink ref="F5" r:id="rId4" display="https://www.digikey.de/de/products/detail/nxp-usa-inc/LM75BD-118/1992993"/>
-    <hyperlink ref="F6" r:id="rId5" display="https://www.digikey.de/de/products/detail/sensirion-ag/SHTC3-TR-2-5KS/8628148"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F9" r:id="rId6" xr:uid="{49CB2F73-DFB1-4F2F-B6A8-61BB545EBA71}"/>
+    <hyperlink ref="F7" r:id="rId7" xr:uid="{1CC8E20B-9A58-4173-88E0-2AB67BE15C1D}"/>
   </hyperlinks>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>